<commit_message>
mark identifier as required in HEI list
</commit_message>
<xml_diff>
--- a/docs/files/Template_HEI_lists.xlsx
+++ b/docs/files/Template_HEI_lists.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="95">
   <si>
     <t xml:space="preserve">agency_id</t>
   </si>
@@ -159,6 +159,7 @@
         <sz val="10"/>
         <rFont val="Arial"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Institution:
 </t>
@@ -168,6 +169,7 @@
         <sz val="9"/>
         <rFont val="Arial"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Official name (in local/official language and script)</t>
     </r>
@@ -194,6 +196,7 @@
         <sz val="9"/>
         <rFont val="Arial"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Institution:
 identifier of this institution – </t>
@@ -204,6 +207,7 @@
         <sz val="9"/>
         <rFont val="Arial"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">please provide WHED identifier</t>
     </r>
@@ -212,6 +216,7 @@
         <sz val="9"/>
         <rFont val="Arial"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve"> if possible, e.g. IAU-123456</t>
     </r>
@@ -226,6 +231,7 @@
         <sz val="9"/>
         <rFont val="Arial"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Institution: 
 details on the source and issuer of the identifier – </t>
@@ -236,6 +242,7 @@
         <sz val="9"/>
         <rFont val="Arial"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">required if this type is not yet known to EQAR</t>
     </r>
@@ -244,6 +251,7 @@
         <sz val="9"/>
         <rFont val="Arial"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve"> – skip for WHED</t>
     </r>
@@ -254,6 +262,7 @@
         <sz val="9"/>
         <rFont val="Arial"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Institution:
 official source (e.g. ministry website, national register, …) proving that this provider has full degree awarding powers in at least one higher education system – </t>
@@ -264,6 +273,7 @@
         <sz val="9"/>
         <rFont val="Arial"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">required if no WHED identifier provided</t>
     </r>
@@ -272,6 +282,7 @@
         <sz val="9"/>
         <rFont val="Arial"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve"> – institution's own website is not accepted</t>
     </r>
@@ -286,6 +297,7 @@
         <sz val="10"/>
         <rFont val="Arial"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Institution legal seat:
 </t>
@@ -295,6 +307,7 @@
         <sz val="9"/>
         <rFont val="Arial"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Country – ISO 3166 (2-letter or 3-letter) code or numerical DEQAR ID</t>
     </r>
@@ -368,9 +381,6 @@
     <t xml:space="preserve">optional</t>
   </si>
   <si>
-    <t xml:space="preserve">recommended</t>
-  </si>
-  <si>
     <t xml:space="preserve">conditionally req.</t>
   </si>
   <si>
@@ -379,6 +389,7 @@
         <sz val="10"/>
         <rFont val="Arial"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">required if </t>
     </r>
@@ -388,6 +399,7 @@
         <sz val="10"/>
         <rFont val="Arial"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">parent_id</t>
     </r>
@@ -396,6 +408,7 @@
         <sz val="10"/>
         <rFont val="Arial"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve"> present</t>
     </r>
@@ -445,6 +458,7 @@
         <sz val="10"/>
         <rFont val="Arial"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Institution DEQARINST ID
 </t>
@@ -455,6 +469,7 @@
         <sz val="10"/>
         <rFont val="Arial"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">(preferred)</t>
     </r>
@@ -529,11 +544,12 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -555,20 +571,29 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="9"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
       <sz val="9"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <i val="true"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -641,12 +666,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -654,23 +683,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -679,18 +696,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -698,39 +707,23 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -918,49 +911,49 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:BY4"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10.62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="23.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="13.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12.51"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="13.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="16.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="15.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="24.47"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="11" style="0" width="13.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="17" style="0" width="14.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="0" width="13.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="0" width="22.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="0" width="13.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="0" width="22.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="26" style="0" width="14.87"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="30" style="0" width="16.95"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="31" min="31" style="0" width="30.46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="13.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="23.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="13.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="13.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="12.51"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="13.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="16.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="15.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="24.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="11" style="1" width="13.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="17" style="1" width="14.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="1" width="13.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="1" width="22.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="1" width="13.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="1" width="22.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="26" style="1" width="14.87"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="30" style="1" width="16.95"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="31" min="31" style="1" width="30.46"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
       <c r="H1" s="3" t="s">
@@ -969,40 +962,40 @@
       <c r="I1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
       <c r="K1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
       <c r="N1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="O1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="P1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="Q1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="R1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="S1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="T1" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="U1" s="3" t="s">
         <v>20</v>
       </c>
       <c r="V1" s="3" t="s">
@@ -1017,16 +1010,16 @@
       <c r="Y1" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AB1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AC1" s="2" t="s">
         <v>28</v>
       </c>
       <c r="AD1" s="3" t="s">
@@ -1035,241 +1028,240 @@
       <c r="AE1" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" s="5"/>
-      <c r="AG1" s="5"/>
-      <c r="AH1" s="5"/>
-      <c r="AI1" s="5"/>
-      <c r="AJ1" s="5"/>
-      <c r="AK1" s="5"/>
-      <c r="AL1" s="5"/>
-      <c r="AM1" s="5"/>
-      <c r="AN1" s="5"/>
-      <c r="AO1" s="5"/>
-      <c r="AP1" s="5"/>
-      <c r="AQ1" s="5"/>
-      <c r="AR1" s="5"/>
-      <c r="AS1" s="5"/>
-      <c r="AT1" s="5"/>
-      <c r="AU1" s="5"/>
-      <c r="AV1" s="5"/>
-      <c r="AW1" s="5"/>
-      <c r="AX1" s="5"/>
-      <c r="AY1" s="5"/>
-      <c r="AZ1" s="5"/>
-      <c r="BA1" s="5"/>
-      <c r="BB1" s="5"/>
-      <c r="BC1" s="5"/>
-      <c r="BD1" s="5"/>
-      <c r="BE1" s="5"/>
-      <c r="BF1" s="5"/>
-      <c r="BG1" s="5"/>
-      <c r="BH1" s="5"/>
-      <c r="BI1" s="5"/>
-      <c r="BJ1" s="5"/>
-      <c r="BK1" s="5"/>
-      <c r="BL1" s="5"/>
-      <c r="BM1" s="5"/>
-      <c r="BN1" s="5"/>
-      <c r="BO1" s="5"/>
-      <c r="BP1" s="5"/>
-      <c r="BQ1" s="5"/>
-      <c r="BR1" s="5"/>
-      <c r="BS1" s="5"/>
-      <c r="BT1" s="5"/>
-      <c r="BU1" s="5"/>
-      <c r="BV1" s="5"/>
-      <c r="BW1" s="5"/>
-      <c r="BX1" s="5"/>
-      <c r="BY1" s="5"/>
+      <c r="AF1" s="4"/>
+      <c r="AG1" s="4"/>
+      <c r="AH1" s="4"/>
+      <c r="AI1" s="4"/>
+      <c r="AJ1" s="4"/>
+      <c r="AK1" s="4"/>
+      <c r="AL1" s="4"/>
+      <c r="AM1" s="4"/>
+      <c r="AN1" s="4"/>
+      <c r="AO1" s="4"/>
+      <c r="AP1" s="4"/>
+      <c r="AQ1" s="4"/>
+      <c r="AR1" s="4"/>
+      <c r="AS1" s="4"/>
+      <c r="AT1" s="4"/>
+      <c r="AU1" s="4"/>
+      <c r="AV1" s="4"/>
+      <c r="AW1" s="4"/>
+      <c r="AX1" s="4"/>
+      <c r="AY1" s="4"/>
+      <c r="AZ1" s="4"/>
+      <c r="BA1" s="4"/>
+      <c r="BB1" s="4"/>
+      <c r="BC1" s="4"/>
+      <c r="BD1" s="4"/>
+      <c r="BE1" s="4"/>
+      <c r="BF1" s="4"/>
+      <c r="BG1" s="4"/>
+      <c r="BH1" s="4"/>
+      <c r="BI1" s="4"/>
+      <c r="BJ1" s="4"/>
+      <c r="BK1" s="4"/>
+      <c r="BL1" s="4"/>
+      <c r="BM1" s="4"/>
+      <c r="BN1" s="4"/>
+      <c r="BO1" s="4"/>
+      <c r="BP1" s="4"/>
+      <c r="BQ1" s="4"/>
+      <c r="BR1" s="4"/>
+      <c r="BS1" s="4"/>
+      <c r="BT1" s="4"/>
+      <c r="BU1" s="4"/>
+      <c r="BV1" s="4"/>
+      <c r="BW1" s="4"/>
+      <c r="BX1" s="4"/>
+      <c r="BY1" s="4"/>
     </row>
     <row r="2" customFormat="false" ht="115.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D2" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="F2" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="G2" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="H2" s="9" t="s">
+      <c r="H2" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="I2" s="9" t="s">
+      <c r="I2" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="J2" s="9" t="s">
+      <c r="J2" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="K2" s="9" t="s">
+      <c r="K2" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="L2" s="7" t="s">
+      <c r="L2" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="M2" s="7" t="s">
+      <c r="M2" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="N2" s="10" t="s">
+      <c r="N2" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="O2" s="9" t="s">
+      <c r="O2" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="P2" s="9" t="s">
+      <c r="P2" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="Q2" s="9" t="s">
+      <c r="Q2" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="R2" s="9" t="s">
+      <c r="R2" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="S2" s="9" t="s">
+      <c r="S2" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="T2" s="9" t="s">
+      <c r="T2" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="U2" s="9" t="s">
+      <c r="U2" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="V2" s="9" t="s">
+      <c r="V2" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="W2" s="11" t="s">
+      <c r="W2" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="X2" s="9" t="s">
+      <c r="X2" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="Y2" s="11" t="s">
+      <c r="Y2" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="Z2" s="6" t="s">
+      <c r="Z2" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="AA2" s="6"/>
-      <c r="AB2" s="6"/>
-      <c r="AC2" s="6"/>
-      <c r="AD2" s="9" t="s">
+      <c r="AA2" s="5"/>
+      <c r="AB2" s="5"/>
+      <c r="AC2" s="5"/>
+      <c r="AD2" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="AE2" s="6" t="s">
+      <c r="AE2" s="5" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="C3" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="D3" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="E3" s="12" t="s">
+      <c r="C3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="E3" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="F3" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="G3" s="15" t="s">
+      <c r="F3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="H3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="I3" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="H3" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="I3" s="16" t="s">
+      <c r="J3" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="K3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="L3" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="M3" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="N3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="O3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="P3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="R3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="S3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="T3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="U3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="V3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="W3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="X3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="Y3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="Z3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="AA3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="AB3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="AC3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="AD3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="AE3" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="J3" s="16" t="s">
-        <v>61</v>
-      </c>
-      <c r="K3" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="L3" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="M3" s="17" t="s">
-        <v>58</v>
-      </c>
-      <c r="N3" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="O3" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="P3" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="Q3" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="R3" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="S3" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="T3" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="U3" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="V3" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="W3" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="X3" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="Y3" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="Z3" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="AA3" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="AB3" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="AC3" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="AD3" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="AE3" s="16" t="s">
-        <v>62</v>
-      </c>
     </row>
-    <row r="4" s="19" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="18"/>
-      <c r="L4" s="18"/>
-      <c r="Q4" s="0"/>
+    <row r="4" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="11"/>
+      <c r="L4" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1292,62 +1284,62 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:BN3"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="18.74"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="26.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="13.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="13.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="8" style="0" width="13.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="12.28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="9.08"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="9.6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="20" width="14.21"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="17" style="0" width="14.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="9.21"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="0" width="17.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="0" width="9.64"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="0" width="40.95"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="18.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="26.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="13.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="1" width="13.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="8" style="1" width="13.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="12.28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="9.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="9.6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="14.21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="17" style="1" width="14.21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="9.21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="17.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="1" width="9.64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="1" width="40.95"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="C1" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="D1" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>66</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="3" t="s">
         <v>2</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="I1" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="K1" s="20" t="s">
-        <v>70</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>69</v>
+      <c r="L1" s="3" t="s">
+        <v>68</v>
       </c>
       <c r="M1" s="3" t="s">
         <v>4</v>
@@ -1358,7 +1350,7 @@
       <c r="O1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="P1" s="3" t="s">
         <v>11</v>
       </c>
       <c r="Q1" s="3" t="s">
@@ -1368,195 +1360,195 @@
         <v>24</v>
       </c>
       <c r="S1" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="T1" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="T1" s="3" t="s">
+      <c r="U1" s="3" t="s">
         <v>72</v>
-      </c>
-      <c r="U1" s="3" t="s">
-        <v>73</v>
       </c>
       <c r="V1" s="3" t="s">
         <v>29</v>
       </c>
       <c r="W1" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="X1" s="4"/>
+      <c r="Y1" s="4"/>
+      <c r="Z1" s="4"/>
+      <c r="AA1" s="4"/>
+      <c r="AB1" s="4"/>
+      <c r="AC1" s="4"/>
+      <c r="AD1" s="4"/>
+      <c r="AE1" s="4"/>
+      <c r="AF1" s="4"/>
+      <c r="AG1" s="4"/>
+      <c r="AH1" s="4"/>
+      <c r="AI1" s="4"/>
+      <c r="AJ1" s="4"/>
+      <c r="AK1" s="4"/>
+      <c r="AL1" s="4"/>
+      <c r="AM1" s="4"/>
+      <c r="AN1" s="4"/>
+      <c r="AO1" s="4"/>
+      <c r="AP1" s="4"/>
+      <c r="AQ1" s="4"/>
+      <c r="AR1" s="4"/>
+      <c r="AS1" s="4"/>
+      <c r="AT1" s="4"/>
+      <c r="AU1" s="4"/>
+      <c r="AV1" s="4"/>
+      <c r="AW1" s="4"/>
+      <c r="AX1" s="4"/>
+      <c r="AY1" s="4"/>
+      <c r="AZ1" s="4"/>
+      <c r="BA1" s="4"/>
+      <c r="BB1" s="4"/>
+      <c r="BC1" s="4"/>
+      <c r="BD1" s="4"/>
+      <c r="BE1" s="4"/>
+      <c r="BF1" s="4"/>
+      <c r="BG1" s="4"/>
+      <c r="BH1" s="4"/>
+      <c r="BI1" s="4"/>
+      <c r="BJ1" s="4"/>
+      <c r="BK1" s="4"/>
+      <c r="BL1" s="4"/>
+      <c r="BM1" s="4"/>
+      <c r="BN1" s="4"/>
+    </row>
+    <row r="2" customFormat="false" ht="135.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="X1" s="5"/>
-      <c r="Y1" s="5"/>
-      <c r="Z1" s="5"/>
-      <c r="AA1" s="5"/>
-      <c r="AB1" s="5"/>
-      <c r="AC1" s="5"/>
-      <c r="AD1" s="5"/>
-      <c r="AE1" s="5"/>
-      <c r="AF1" s="5"/>
-      <c r="AG1" s="5"/>
-      <c r="AH1" s="5"/>
-      <c r="AI1" s="5"/>
-      <c r="AJ1" s="5"/>
-      <c r="AK1" s="5"/>
-      <c r="AL1" s="5"/>
-      <c r="AM1" s="5"/>
-      <c r="AN1" s="5"/>
-      <c r="AO1" s="5"/>
-      <c r="AP1" s="5"/>
-      <c r="AQ1" s="5"/>
-      <c r="AR1" s="5"/>
-      <c r="AS1" s="5"/>
-      <c r="AT1" s="5"/>
-      <c r="AU1" s="5"/>
-      <c r="AV1" s="5"/>
-      <c r="AW1" s="5"/>
-      <c r="AX1" s="5"/>
-      <c r="AY1" s="5"/>
-      <c r="AZ1" s="5"/>
-      <c r="BA1" s="5"/>
-      <c r="BB1" s="5"/>
-      <c r="BC1" s="5"/>
-      <c r="BD1" s="5"/>
-      <c r="BE1" s="5"/>
-      <c r="BF1" s="5"/>
-      <c r="BG1" s="5"/>
-      <c r="BH1" s="5"/>
-      <c r="BI1" s="5"/>
-      <c r="BJ1" s="5"/>
-      <c r="BK1" s="5"/>
-      <c r="BL1" s="5"/>
-      <c r="BM1" s="5"/>
-      <c r="BN1" s="5"/>
-    </row>
-    <row r="2" customFormat="false" ht="137.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="8" t="s">
+      <c r="B2" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="C2" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="D2" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="E2" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="F2" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="G2" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="G2" s="7" t="s">
+      <c r="H2" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="H2" s="8" t="s">
+      <c r="I2" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="I2" s="8" t="s">
+      <c r="J2" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="J2" s="8" t="s">
+      <c r="K2" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="L2" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="M2" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="K2" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="L2" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="M2" s="7" t="s">
+      <c r="N2" s="6"/>
+      <c r="O2" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="N2" s="7"/>
-      <c r="O2" s="7" t="s">
+      <c r="P2" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="P2" s="8" t="s">
+      <c r="Q2" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="Q2" s="7" t="s">
+      <c r="R2" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="R2" s="7" t="s">
+      <c r="S2" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="S2" s="7" t="s">
+      <c r="T2" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="T2" s="7" t="s">
+      <c r="U2" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="U2" s="7" t="s">
+      <c r="V2" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="V2" s="7" t="s">
+      <c r="W2" s="6" t="s">
         <v>93</v>
-      </c>
-      <c r="W2" s="7" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="21" t="s">
-        <v>95</v>
-      </c>
-      <c r="B3" s="21"/>
-      <c r="C3" s="21"/>
-      <c r="D3" s="21"/>
-      <c r="E3" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="F3" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="G3" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="H3" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="I3" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="J3" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="K3" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="L3" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="M3" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="N3" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="O3" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="P3" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="Q3" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="R3" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="S3" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="T3" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="U3" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="V3" s="22" t="s">
-        <v>59</v>
-      </c>
-      <c r="W3" s="22" t="s">
+      <c r="A3" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="G3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="H3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="I3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="J3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="K3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="L3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="M3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="N3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="O3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="P3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="R3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="S3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="T3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="U3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="V3" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="W3" s="14" t="s">
         <v>59</v>
       </c>
     </row>

</xml_diff>